<commit_message>
refactor(excel): eliminar hojas README y LOG del libro
- README eliminada: contenido duplicado con README.md del repo
- LOG eliminada: contenido duplicado con docs/changelog/CHANGELOG.md
- 6 hojas funcionales intactas (Configuración, Ingresos, Gastos,
  Pagos, Motor, Dashboard)
- Validación: 6 tablas, 13 referencias Motor→Dashboard y
  6 validaciones de datos sin cambios
</commit_message>
<xml_diff>
--- a/product/excel/OpenFinanceKit.xlsx
+++ b/product/excel/OpenFinanceKit.xlsx
@@ -7,14 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="LOG" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Configuración" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Ingresos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gastos" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Pagos" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Motor" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Dashboard" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Configuración" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ingresos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gastos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Pagos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Motor" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Dashboard" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -813,333 +811,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F3864"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>OpenFinanceKit — MVP v0.1.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Sistema de gestión financiera personal</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>¿Qué es OpenFinanceKit?</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>OpenFinanceKit es un sistema para administrar finanzas personales.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Permite registrar ingresos, gastos y pagos, calcular el estado financiero</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>del mes y visualizar un resumen general en el Dashboard.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Hojas del libro</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Hoja</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Descripción</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>README</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Este archivo. Descripción y guía de uso.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>LOG</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Historial de cambios del libro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Configuración</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Categorías, cuentas y parámetros. No modificar sin criterio.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Ingresos</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Registra todos tus ingresos. Solo datos, sin fórmulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Gastos</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Registra todos tus gastos. Solo datos, sin fórmulas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>Pagos</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Pagos programados y su estado (Pendiente/Pagado/Vencido).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Motor</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Realiza TODOS los cálculos. No editar directamente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Resumen visual. Solo lectura.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Reglas de uso</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>RN-001  Configuración es la única fuente de datos maestros.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>RN-002  Motor es la única hoja autorizada para realizar cálculos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>RN-003  Dashboard únicamente visualiza información.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>RN-004  Las hojas de captura (Ingresos, Gastos, Pagos) solo almacenan datos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>RN-005  Las listas desplegables obtienen sus valores desde Configuración.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>RN-006  Las tablas permiten agregar filas sin modificar fórmulas.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="A25:F25"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="007030A0"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>LOG — Historial de cambios</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Versión</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Fecha</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Sprint</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Autor</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Descripción</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>v0.1.0</t>
-        </is>
-      </c>
-      <c r="B4" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="inlineStr">
-        <is>
-          <t>Gustavo Echeverría</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="inlineStr">
-        <is>
-          <t>Creación del MVP — 8 hojas, 6 tablas, Motor y Dashboard</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <tabColor rgb="00ED7D31"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1390,7 +1061,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0070AD47"/>
@@ -1530,7 +1201,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00FF0000"/>
@@ -1670,7 +1341,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00FFC000"/>
@@ -1814,7 +1485,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007030A0"/>
@@ -2065,8 +1736,8 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A14:B14"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A14:B14"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="D9:E9"/>
@@ -2083,7 +1754,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0000B0F0"/>

</xml_diff>

<commit_message>
feat(excel): MVP final — 6 hojas funcionales con Motor y Dashboard
- Configuración: tblCategorias, tblCuentas (val ≥0), tblParametros
- Ingresos: tblIngresos + validaciones (categoría, cuenta, fecha, valor)
- Gastos: tblGastos + validaciones (categoría, cuenta, fecha, valor)
- Pagos: tblPagos + validaciones (estado, fecha, valor)
- Motor: 10 fórmulas (ingresos/gastos mes, balance, saldo actual,
  pendiente, vencido, pagado, disponible restante, % gastado)
- Dashboard: 6 indicadores desde Motor sin fórmulas propias
- SDD: .kiro/specs/feature-excel-mvp-final.md
- 8/8 criterios de aceptación validados
</commit_message>
<xml_diff>
--- a/product/excel/OpenFinanceKit.xlsx
+++ b/product/excel/OpenFinanceKit.xlsx
@@ -21,11 +21,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,11 +38,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
     <font>
@@ -66,13 +62,13 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="20"/>
+      <sz val="16"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00444444"/>
-      <sz val="12"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="16"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -89,47 +85,11 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00C55A11"/>
       <sz val="16"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00375623"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00C55A11"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00888888"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="15">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -139,16 +99,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F9F9F9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -173,7 +123,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C00000"/>
+        <fgColor rgb="00DDEEFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -188,17 +138,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEEFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F7FBFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -228,110 +168,61 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="14" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="166" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <font>
         <b val="1"/>
@@ -347,6 +238,18 @@
       <font>
         <b val="1"/>
         <color rgb="00C00000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00C00000"/>
+        <sz val="16"/>
       </font>
       <fill>
         <patternFill patternType="solid">
@@ -428,8 +331,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblCategorias" displayName="tblCategorias" ref="A1:C11" headerRowCount="1">
-  <autoFilter ref="A1:C11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblCategorias" displayName="tblCategorias" ref="A1:C6" headerRowCount="1">
+  <autoFilter ref="A1:C6"/>
   <tableColumns count="3">
     <tableColumn id="1" name="CategoriaID"/>
     <tableColumn id="2" name="Nombre"/>
@@ -440,8 +343,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblCuentas" displayName="tblCuentas" ref="A13:C16" headerRowCount="1">
-  <autoFilter ref="A13:C16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblCuentas" displayName="tblCuentas" ref="A8:C11" headerRowCount="1">
+  <autoFilter ref="A8:C11"/>
   <tableColumns count="3">
     <tableColumn id="1" name="CuentaID"/>
     <tableColumn id="2" name="Nombre"/>
@@ -452,8 +355,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblParametros" displayName="tblParametros" ref="A18:B21" headerRowCount="1">
-  <autoFilter ref="A18:B21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblParametros" displayName="tblParametros" ref="A13:B16" headerRowCount="1">
+  <autoFilter ref="A13:B16"/>
   <tableColumns count="2">
     <tableColumn id="1" name="Parametro"/>
     <tableColumn id="2" name="Valor"/>
@@ -463,8 +366,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblIngresos" displayName="tblIngresos" ref="A1:F3" headerRowCount="1">
-  <autoFilter ref="A1:F3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblIngresos" displayName="tblIngresos" ref="A1:F2" headerRowCount="1">
+  <autoFilter ref="A1:F2"/>
   <tableColumns count="6">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Fecha"/>
@@ -478,8 +381,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblGastos" displayName="tblGastos" ref="A1:F3" headerRowCount="1">
-  <autoFilter ref="A1:F3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblGastos" displayName="tblGastos" ref="A1:F2" headerRowCount="1">
+  <autoFilter ref="A1:F2"/>
   <tableColumns count="6">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Fecha"/>
@@ -796,12 +699,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -835,37 +738,19 @@
           <t>Ingreso</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Efectivo</t>
-        </is>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Freelance</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Banco</t>
         </is>
       </c>
     </row>
@@ -883,33 +768,21 @@
           <t>Ingreso</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Alimentación</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Gasto</t>
         </is>
       </c>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -925,194 +798,118 @@
           <t>Gasto</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>tblParametros</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>CuentaID</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>SaldoInicial</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Banco</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Parametro</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>MesActual</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>2026-08</t>
         </is>
       </c>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Moneda</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>
       </c>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>CuentaID</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Nombre</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>SaldoInicial</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Efectivo</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Banco</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>Parametro</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>MesActual</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Moneda</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C2:C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Ingreso,Gasto"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C9:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1131,15 +928,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1178,7 +975,7 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
@@ -1193,40 +990,12 @@
           <t>Banco</t>
         </is>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="4" t="n">
         <v>3500</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Sueldo agosto</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Freelance</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Efectivo</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>500</v>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Proyecto web</t>
         </is>
       </c>
     </row>
@@ -1238,10 +1007,10 @@
     <dataValidation sqref="D2:D10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=tblCuentas[Nombre]</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
+    <dataValidation sqref="B2:B10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="date" operator="greaterThan">
       <formula1>DATE(2000,1,1)</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="greaterThan">
+    <dataValidation sqref="E2:E10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="decimal" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -1259,15 +1028,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1306,7 +1075,7 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
@@ -1321,40 +1090,12 @@
           <t>Efectivo</t>
         </is>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="4" t="n">
         <v>120</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Supermercado</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Transporte</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Efectivo</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Gasolina</t>
         </is>
       </c>
     </row>
@@ -1366,10 +1107,10 @@
     <dataValidation sqref="D2:D10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=tblCuentas[Nombre]</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
+    <dataValidation sqref="B2:B10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="date" operator="greaterThan">
       <formula1>DATE(2000,1,1)</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="greaterThan">
+    <dataValidation sqref="E2:E10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="decimal" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -1390,11 +1131,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1433,12 +1174,12 @@
           <t>Internet</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="D2" s="4" t="n">
         <v>45</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1448,23 +1189,23 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Seguro</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3" s="4" t="n">
         <v>120</v>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -1479,12 +1220,12 @@
           <t>Gimnasio</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="4" t="n">
         <v>35</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1498,10 +1239,10 @@
     <dataValidation sqref="E2:E10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pendiente,Pagado,Vencido"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
+    <dataValidation sqref="C2:C10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="date" operator="greaterThan">
       <formula1>DATE(2000,1,1)</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="greaterThan">
+    <dataValidation sqref="D2:D10000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="decimal" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -1519,239 +1260,168 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="3" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Resumen del mes</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
-        <is>
-          <t>Ingresos por categoría</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Total Ingresos del mes</t>
-        </is>
-      </c>
-      <c r="B2" s="13">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Ingresos del mes</t>
+        </is>
+      </c>
+      <c r="B2" s="9">
         <f>SUMPRODUCT((YEAR(tblIngresos[Fecha])=YEAR(DATEVALUE(INDEX(tblParametros[Valor],MATCH("MesActual",tblParametros[Parametro],0))&amp;"-01")))*(MONTH(tblIngresos[Fecha])=MONTH(DATEVALUE(INDEX(tblParametros[Valor],MATCH("MesActual",tblParametros[Parametro],0))&amp;"-01")))*tblIngresos[Valor])</f>
         <v/>
       </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>Sueldo</t>
-        </is>
-      </c>
-      <c r="E2" s="13">
-        <f>SUMIF(tblIngresos[Categoria],"Sueldo",tblIngresos[Valor])</f>
-        <v/>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Total Gastos del mes</t>
-        </is>
-      </c>
-      <c r="B3" s="13">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Gastos del mes</t>
+        </is>
+      </c>
+      <c r="B3" s="9">
         <f>SUMPRODUCT((YEAR(tblGastos[Fecha])=YEAR(DATEVALUE(INDEX(tblParametros[Valor],MATCH("MesActual",tblParametros[Parametro],0))&amp;"-01")))*(MONTH(tblGastos[Fecha])=MONTH(DATEVALUE(INDEX(tblParametros[Valor],MATCH("MesActual",tblParametros[Parametro],0))&amp;"-01")))*tblGastos[Valor])</f>
         <v/>
       </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>Freelance</t>
-        </is>
-      </c>
-      <c r="E3" s="13">
-        <f>SUMIF(tblIngresos[Categoria],"Freelance",tblIngresos[Valor])</f>
-        <v/>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Balance del mes</t>
         </is>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="9">
         <f>B2-B3</f>
         <v/>
       </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Otros ingresos</t>
-        </is>
-      </c>
-      <c r="E4" s="13">
-        <f>SUMIF(tblIngresos[Categoria],"Otros ingresos",tblIngresos[Valor])</f>
-        <v/>
-      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>Saldos por cuenta</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>Gastos por categoría</t>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Saldo actual</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Saldo — Efectivo</t>
-        </is>
-      </c>
-      <c r="B7" s="13">
-        <f>SUMIF(tblCuentas[Nombre],"Efectivo",tblCuentas[SaldoInicial])+SUMIF(tblIngresos[Cuenta],"Efectivo",tblIngresos[Valor])-SUMIF(tblGastos[Cuenta],"Efectivo",tblGastos[Valor])</f>
-        <v/>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Alimentación</t>
-        </is>
-      </c>
-      <c r="E7" s="13">
-        <f>SUMIF(tblGastos[Categoria],"Alimentación",tblGastos[Valor])</f>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Total Ingresos (histórico)</t>
+        </is>
+      </c>
+      <c r="B7" s="9">
+        <f>SUM(tblIngresos[Valor])</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Saldo — Banco</t>
-        </is>
-      </c>
-      <c r="B8" s="13">
-        <f>SUMIF(tblCuentas[Nombre],"Banco",tblCuentas[SaldoInicial])+SUMIF(tblIngresos[Cuenta],"Banco",tblIngresos[Valor])-SUMIF(tblGastos[Cuenta],"Banco",tblGastos[Valor])</f>
-        <v/>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>Transporte</t>
-        </is>
-      </c>
-      <c r="E8" s="13">
-        <f>SUMIF(tblGastos[Categoria],"Transporte",tblGastos[Valor])</f>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Total Gastos (histórico)</t>
+        </is>
+      </c>
+      <c r="B8" s="9">
+        <f>SUM(tblGastos[Valor])</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Saldo — Tarjeta</t>
-        </is>
-      </c>
-      <c r="B9" s="13">
-        <f>SUMIF(tblCuentas[Nombre],"Tarjeta",tblCuentas[SaldoInicial])+SUMIF(tblIngresos[Cuenta],"Tarjeta",tblIngresos[Valor])-SUMIF(tblGastos[Cuenta],"Tarjeta",tblGastos[Valor])</f>
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Saldo actual</t>
+        </is>
+      </c>
+      <c r="B9" s="9">
+        <f>SUM(tblCuentas[SaldoInicial])+B7-B8</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>Totales generales</t>
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Pagos</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Total Ingresos (histórico)</t>
-        </is>
-      </c>
-      <c r="B12" s="13">
-        <f>SUM(tblIngresos[Valor])</f>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente de pago</t>
+        </is>
+      </c>
+      <c r="B12" s="9">
+        <f>SUMIF(tblPagos[Estado],"Pendiente",tblPagos[Valor])</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Total Gastos (histórico)</t>
-        </is>
-      </c>
-      <c r="B13" s="13">
-        <f>SUM(tblGastos[Valor])</f>
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Total vencido</t>
+        </is>
+      </c>
+      <c r="B13" s="10">
+        <f>SUMIF(tblPagos[Estado],"Vencido",tblPagos[Valor])</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Saldo actual total</t>
-        </is>
-      </c>
-      <c r="B14" s="13">
-        <f>SUM(tblCuentas[SaldoInicial])+B12-B13</f>
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Total pagado</t>
+        </is>
+      </c>
+      <c r="B14" s="9">
+        <f>SUMIF(tblPagos[Estado],"Pagado",tblPagos[Valor])</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>Pagos</t>
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Indicadores clave</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Pendiente de pago</t>
-        </is>
-      </c>
-      <c r="B17" s="13">
-        <f>SUMIF(tblPagos[Estado],"Pendiente",tblPagos[Valor])</f>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Disponible restante</t>
+        </is>
+      </c>
+      <c r="B17" s="9">
+        <f>B9-B12</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Total vencido</t>
-        </is>
-      </c>
-      <c r="B18" s="15">
-        <f>SUMIF(tblPagos[Estado],"Vencido",tblPagos[Valor])</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Total pagado</t>
-        </is>
-      </c>
-      <c r="B19" s="13">
-        <f>SUMIF(tblPagos[Estado],"Pagado",tblPagos[Valor])</f>
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>% Gastado</t>
+        </is>
+      </c>
+      <c r="B18" s="12">
+        <f>IFERROR(B3/B2,0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="D6:E6"/>
+  <mergeCells count="4">
+    <mergeCell ref="A11:B11"/>
     <mergeCell ref="A16:B16"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A6:B6"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A6:B6"/>
   </mergeCells>
   <conditionalFormatting sqref="B4">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
@@ -1759,6 +1429,14 @@
     </cfRule>
     <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
       <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B18">
+    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="1">
+      <formula>0.8</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="lessThanOrEqual" dxfId="0">
+      <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1772,257 +1450,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
-        <is>
-          <t>OpenFinanceKit — Dashboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="17">
-        <f>CONCATENATE("Período: ",IFERROR(INDEX(tblParametros[Valor],MATCH("MesActual",tblParametros[Parametro],0)),"N/A"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>💰 INGRESOS</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>💸 GASTOS</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>📊 BALANCE</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>⏳ PENDIENTE</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>🚨 VENCIDO</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="18">
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="13">
+        <f>CONCATENATE("OpenFinanceKit — ",INDEX(tblParametros[Valor],MATCH("MesActual",tblParametros[Parametro],0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Saldo actual</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Ingresos del mes</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Gastos del mes</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Pendiente por pagar</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="14">
+        <f>Motor!B9</f>
+        <v/>
+      </c>
+      <c r="B4" s="15">
         <f>Motor!B2</f>
         <v/>
       </c>
-      <c r="B5" s="19">
+      <c r="D4" s="16">
         <f>Motor!B3</f>
         <v/>
       </c>
-      <c r="C5" s="20">
-        <f>Motor!B4</f>
-        <v/>
-      </c>
-      <c r="D5" s="21">
+      <c r="E4" s="17">
+        <f>Motor!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Disponible restante</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>% Gastado</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="15">
         <f>Motor!B17</f>
         <v/>
       </c>
-      <c r="E5" s="19">
+      <c r="B7" s="18">
         <f>Motor!B18</f>
         <v/>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
-        <is>
-          <t>Saldos por cuenta</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Cuenta</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="inlineStr">
-        <is>
-          <t>Saldo Inicial</t>
-        </is>
-      </c>
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>Entradas</t>
-        </is>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
-        <is>
-          <t>Salidas</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>Saldo Actual</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="23" t="inlineStr">
-        <is>
-          <t>Efectivo</t>
-        </is>
-      </c>
-      <c r="B9" s="24">
-        <f>SUMIF(tblCuentas[Nombre],"Efectivo",tblCuentas[SaldoInicial])</f>
-        <v/>
-      </c>
-      <c r="C9" s="24">
-        <f>SUMIF(tblIngresos[Cuenta],"Efectivo",tblIngresos[Valor])</f>
-        <v/>
-      </c>
-      <c r="D9" s="24">
-        <f>SUMIF(tblGastos[Cuenta],"Efectivo",tblGastos[Valor])</f>
-        <v/>
-      </c>
-      <c r="E9" s="24">
-        <f>Motor!B7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="25" t="inlineStr">
-        <is>
-          <t>Banco</t>
-        </is>
-      </c>
-      <c r="B10" s="26">
-        <f>SUMIF(tblCuentas[Nombre],"Banco",tblCuentas[SaldoInicial])</f>
-        <v/>
-      </c>
-      <c r="C10" s="26">
-        <f>SUMIF(tblIngresos[Cuenta],"Banco",tblIngresos[Valor])</f>
-        <v/>
-      </c>
-      <c r="D10" s="26">
-        <f>SUMIF(tblGastos[Cuenta],"Banco",tblGastos[Valor])</f>
-        <v/>
-      </c>
-      <c r="E10" s="26">
-        <f>Motor!B8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="23" t="inlineStr">
-        <is>
-          <t>Tarjeta</t>
-        </is>
-      </c>
-      <c r="B11" s="24">
-        <f>SUMIF(tblCuentas[Nombre],"Tarjeta",tblCuentas[SaldoInicial])</f>
-        <v/>
-      </c>
-      <c r="C11" s="24">
-        <f>SUMIF(tblIngresos[Cuenta],"Tarjeta",tblIngresos[Valor])</f>
-        <v/>
-      </c>
-      <c r="D11" s="24">
-        <f>SUMIF(tblGastos[Cuenta],"Tarjeta",tblGastos[Valor])</f>
-        <v/>
-      </c>
-      <c r="E11" s="24">
-        <f>Motor!B9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="22" t="inlineStr">
-        <is>
-          <t>Resumen del mes</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Total Ingresos del mes</t>
-        </is>
-      </c>
-      <c r="B14" s="27">
-        <f>Motor!B2</f>
-        <v/>
-      </c>
-      <c r="C14" s="28" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>Total Gastos del mes</t>
-        </is>
-      </c>
-      <c r="B15" s="29">
-        <f>Motor!B3</f>
-        <v/>
-      </c>
-      <c r="C15" s="30" t="n"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Balance del mes</t>
-        </is>
-      </c>
-      <c r="B16" s="31">
-        <f>Motor!B4</f>
-        <v/>
-      </c>
-      <c r="C16" s="32" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Pendiente de pago</t>
-        </is>
-      </c>
-      <c r="B17" s="33">
-        <f>Motor!B17</f>
-        <v/>
-      </c>
-      <c r="C17" s="34" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Total vencido</t>
-        </is>
-      </c>
-      <c r="B18" s="29">
-        <f>Motor!B18</f>
-        <v/>
-      </c>
-      <c r="C18" s="30" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="35" t="inlineStr">
-        <is>
-          <t>⚠️ Solo lectura. No editar. Los datos provienen del Motor.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A4">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>